<commit_message>
refactor: organize single Next.js app at repository root
</commit_message>
<xml_diff>
--- a/docs/business/紬_事業の中身.xlsx
+++ b/docs/business/紬_事業の中身.xlsx
@@ -567,7 +567,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -664,7 +664,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -761,7 +761,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -842,7 +842,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -923,7 +923,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1004,7 +1004,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1069,7 +1069,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1134,7 +1134,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1199,7 +1199,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1264,7 +1264,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1377,7 +1377,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1442,7 +1442,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1523,7 +1523,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -1620,7 +1620,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2228,7 +2228,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2293,7 +2293,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2358,7 +2358,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2423,7 +2423,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2488,7 +2488,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2553,7 +2553,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2618,7 +2618,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2683,7 +2683,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -2758,7 +2758,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+          <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
         </r>
         <r>
           <rPr>
@@ -3415,7 +3415,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">site/src/content/prices.ts</t>
+      <t xml:space="preserve">src/content/prices.ts</t>
     </r>
   </si>
   <si>
@@ -3771,7 +3771,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">site/public/verify-report.json </t>
+      <t xml:space="preserve">public/verify-report.json </t>
     </r>
     <r>
       <rPr>
@@ -4930,7 +4930,7 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">: site/src/content/prices.ts / 2026-09-14</t>
+      <t xml:space="preserve">: src/content/prices.ts / 2026-09-14</t>
     </r>
     <r>
       <rPr>

</xml_diff>

<commit_message>
fix: present production-only pricing without mandatory maintenance
</commit_message>
<xml_diff>
--- a/docs/business/紬_事業の中身.xlsx
+++ b/docs/business/紬_事業の中身.xlsx
@@ -3717,7 +3717,7 @@
     <row r="3" ht="48" customHeight="1" s="64">
       <c r="A3" s="97" t="inlineStr">
         <is>
-          <t>参考価格の比較です。役務は同一ではありません。「守る」は通常変更なし、比較先は月5回の更新を含みます。</t>
+          <t>紬は保守契約なし・制作のみ。外部実費は別途。比較先は月5回の更新を含み、紬は自分で管理します。</t>
         </is>
       </c>
       <c r="B3" s="98" t="n"/>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="C5" s="67" t="inlineStr">
         <is>
-          <t>月次保守</t>
+          <t>任意の月次支援</t>
         </is>
       </c>
       <c r="D5" s="67" t="inlineStr">
@@ -3775,8 +3775,8 @@
         <v>79800</v>
       </c>
       <c r="C6" s="101" t="n">
-        <f>料金レバー!$C$20</f>
-        <v>3900</v>
+        <f>料金レバー!$C$23</f>
+        <v>0</v>
       </c>
       <c r="D6" s="101" t="n">
         <f>料金レバー!$C$16</f>
@@ -3784,7 +3784,7 @@
       </c>
       <c r="E6" s="101" t="n">
         <f>B6+(C6+D6)*料金レバー!$C$25</f>
-        <v>346200</v>
+        <v>205800</v>
       </c>
       <c r="F6" s="101" t="n">
         <f>料金レバー!$C$29+料金レバー!$C$26*料金レバー!$C$25</f>
@@ -3792,7 +3792,7 @@
       </c>
       <c r="G6" s="101" t="n">
         <f>E6-F6</f>
-        <v>-11600</v>
+        <v>-152000</v>
       </c>
     </row>
     <row r="7" ht="63.75" customHeight="1" s="64">
@@ -3806,8 +3806,8 @@
         <v>198000</v>
       </c>
       <c r="C7" s="101" t="n">
-        <f>料金レバー!$C$20</f>
-        <v>3900</v>
+        <f>料金レバー!$C$23</f>
+        <v>0</v>
       </c>
       <c r="D7" s="101" t="n">
         <f>料金レバー!$C$16</f>
@@ -3815,7 +3815,7 @@
       </c>
       <c r="E7" s="101" t="n">
         <f>B7+(C7+D7)*料金レバー!$C$25</f>
-        <v>464400</v>
+        <v>324000</v>
       </c>
       <c r="F7" s="101" t="n">
         <f>料金レバー!$C$29+料金レバー!$C$27*料金レバー!$C$25</f>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="G7" s="101" t="n">
         <f>E7-F7</f>
-        <v>-73400</v>
+        <v>-213800</v>
       </c>
     </row>
     <row r="8" ht="63.75" customHeight="1" s="64">
@@ -3837,8 +3837,8 @@
         <v>398000</v>
       </c>
       <c r="C8" s="101" t="n">
-        <f>料金レバー!$C$20</f>
-        <v>3900</v>
+        <f>料金レバー!$C$23</f>
+        <v>0</v>
       </c>
       <c r="D8" s="101" t="n">
         <f>料金レバー!$C$16</f>
@@ -3846,7 +3846,7 @@
       </c>
       <c r="E8" s="101" t="n">
         <f>B8+(C8+D8)*料金レバー!$C$25</f>
-        <v>664400</v>
+        <v>524000</v>
       </c>
       <c r="F8" s="101" t="n">
         <f>料金レバー!$C$29+料金レバー!$C$28*料金レバー!$C$25</f>
@@ -3854,7 +3854,7 @@
       </c>
       <c r="G8" s="101" t="n">
         <f>E8-F8</f>
-        <v>-53400</v>
+        <v>-193800</v>
       </c>
     </row>
     <row r="10" ht="63.75" customHeight="1" s="64">
@@ -3891,7 +3891,7 @@
     <row r="12" ht="64.5" customHeight="1" s="64">
       <c r="A12" s="97" t="inlineStr">
         <is>
-          <t>すべて税別。外部費は仮定であり実見積もりに置換。最安値や効果の保証ではありません。情報を育てるは受付準備中。最低契約6か月、36か月後の継続・譲渡は比較先の条件を確認。</t>
+          <t>すべて税別。紬の制作は79,800円から、保守契約なしなら紬への月額0円。外部費は概算。育てるは受付準備中。比較先は最低6か月、36か月後の継続・譲渡条件を確認。</t>
         </is>
       </c>
       <c r="B12" s="98" t="n"/>
@@ -6255,7 +6255,7 @@
     <row r="3" ht="48" customHeight="1" s="64">
       <c r="A3" s="97" t="inlineStr">
         <is>
-          <t>参考価格の比較です。役務は同一ではありません。「守る」は通常変更なし、比較先は月5回の更新を含みます。</t>
+          <t>紬は保守契約なし・制作のみ。外部実費は別途。比較先は月5回の更新を含み、紬は自分で管理します。</t>
         </is>
       </c>
       <c r="B3" s="98" t="n"/>
@@ -6278,7 +6278,7 @@
       </c>
       <c r="C5" s="67" t="inlineStr">
         <is>
-          <t>月次保守</t>
+          <t>任意の月次支援</t>
         </is>
       </c>
       <c r="D5" s="67" t="inlineStr">
@@ -6313,8 +6313,8 @@
         <v>79800</v>
       </c>
       <c r="C6" s="101" t="n">
-        <f>料金レバー!$C$20</f>
-        <v>3900</v>
+        <f>料金レバー!$C$23</f>
+        <v>0</v>
       </c>
       <c r="D6" s="101" t="n">
         <f>料金レバー!$C$16</f>
@@ -6322,7 +6322,7 @@
       </c>
       <c r="E6" s="101" t="n">
         <f>B6+(C6+D6)*料金レバー!$C$25</f>
-        <v>346200</v>
+        <v>205800</v>
       </c>
       <c r="F6" s="101" t="n">
         <f>料金レバー!$C$29+料金レバー!$C$26*料金レバー!$C$25</f>
@@ -6330,7 +6330,7 @@
       </c>
       <c r="G6" s="101" t="n">
         <f>E6-F6</f>
-        <v>-11600</v>
+        <v>-152000</v>
       </c>
     </row>
     <row r="7" ht="63.75" customHeight="1" s="64">
@@ -6344,8 +6344,8 @@
         <v>198000</v>
       </c>
       <c r="C7" s="101" t="n">
-        <f>料金レバー!$C$20</f>
-        <v>3900</v>
+        <f>料金レバー!$C$23</f>
+        <v>0</v>
       </c>
       <c r="D7" s="101" t="n">
         <f>料金レバー!$C$16</f>
@@ -6353,7 +6353,7 @@
       </c>
       <c r="E7" s="101" t="n">
         <f>B7+(C7+D7)*料金レバー!$C$25</f>
-        <v>464400</v>
+        <v>324000</v>
       </c>
       <c r="F7" s="101" t="n">
         <f>料金レバー!$C$29+料金レバー!$C$27*料金レバー!$C$25</f>
@@ -6361,7 +6361,7 @@
       </c>
       <c r="G7" s="101" t="n">
         <f>E7-F7</f>
-        <v>-73400</v>
+        <v>-213800</v>
       </c>
     </row>
     <row r="8" ht="63.75" customHeight="1" s="64">
@@ -6375,8 +6375,8 @@
         <v>398000</v>
       </c>
       <c r="C8" s="101" t="n">
-        <f>料金レバー!$C$20</f>
-        <v>3900</v>
+        <f>料金レバー!$C$23</f>
+        <v>0</v>
       </c>
       <c r="D8" s="101" t="n">
         <f>料金レバー!$C$16</f>
@@ -6384,7 +6384,7 @@
       </c>
       <c r="E8" s="101" t="n">
         <f>B8+(C8+D8)*料金レバー!$C$25</f>
-        <v>664400</v>
+        <v>524000</v>
       </c>
       <c r="F8" s="101" t="n">
         <f>料金レバー!$C$29+料金レバー!$C$28*料金レバー!$C$25</f>
@@ -6392,7 +6392,7 @@
       </c>
       <c r="G8" s="101" t="n">
         <f>E8-F8</f>
-        <v>-53400</v>
+        <v>-193800</v>
       </c>
     </row>
     <row r="10" ht="63.75" customHeight="1" s="64">
@@ -6429,7 +6429,7 @@
     <row r="12" ht="64.5" customHeight="1" s="64">
       <c r="A12" s="97" t="inlineStr">
         <is>
-          <t>すべて税別。外部費は仮定であり実見積もりに置換。最安値や効果の保証ではありません。情報を育てるは受付準備中。最低契約6か月、36か月後の継続・譲渡は比較先の条件を確認。</t>
+          <t>すべて税別。紬の制作は79,800円から、保守契約なしなら紬への月額0円。外部費は概算。育てるは受付準備中。比較先は最低6か月、36か月後の継続・譲渡条件を確認。</t>
         </is>
       </c>
       <c r="B12" s="98" t="n"/>

</xml_diff>